<commit_message>
Raise demo activity so two of the four standards read green
All four daily averages landed under target in the demo data, so the
standards block on the KPI Dashboard was entirely red — no way to show the
green state while recording, and a bleak first impression of the sheet.

Reels and opener DMs now average above target, stories and follow-ups
below. That also gives the video a real coaching line to deliver: posting
and openers are holding, stories and follow-ups are where the gap is.

Template values are unchanged — this only affects the recording copy.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ByBdvAsLbjH7ye5fUDygK8
</commit_message>
<xml_diff>
--- a/docs/The_Called_Client_Tracker_DEMO.xlsx
+++ b/docs/The_Called_Client_Tracker_DEMO.xlsx
@@ -2390,13 +2390,13 @@
         <v/>
       </c>
       <c r="C4" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E4" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F4" s="27" t="n">
         <v>9</v>
@@ -2449,13 +2449,13 @@
         <v/>
       </c>
       <c r="C5" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="27" t="n">
         <v>31</v>
       </c>
       <c r="E5" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F5" s="27" t="n">
         <v>9</v>
@@ -2504,13 +2504,13 @@
         <v/>
       </c>
       <c r="C6" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="27" t="n">
         <v>28</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F6" s="27" t="n">
         <v>9</v>
@@ -2559,13 +2559,13 @@
         <v/>
       </c>
       <c r="C7" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="27" t="n">
         <v>34</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F7" s="27" t="n">
         <v>10</v>
@@ -2614,13 +2614,13 @@
         <v/>
       </c>
       <c r="C8" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E8" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F8" s="27" t="n">
         <v>13</v>
@@ -2779,13 +2779,13 @@
         <v/>
       </c>
       <c r="C11" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="27" t="n">
         <v>35</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F11" s="27" t="n">
         <v>13</v>
@@ -2834,13 +2834,13 @@
         <v/>
       </c>
       <c r="C12" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" s="27" t="n">
         <v>35</v>
       </c>
       <c r="E12" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F12" s="27" t="n">
         <v>9</v>
@@ -2889,13 +2889,13 @@
         <v/>
       </c>
       <c r="C13" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" s="27" t="n">
         <v>33</v>
       </c>
       <c r="E13" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F13" s="27" t="n">
         <v>12</v>
@@ -2944,13 +2944,13 @@
         <v/>
       </c>
       <c r="C14" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D14" s="27" t="n">
         <v>29</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F14" s="27" t="n">
         <v>11</v>
@@ -2999,13 +2999,13 @@
         <v/>
       </c>
       <c r="C15" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15" s="27" t="n">
         <v>33</v>
       </c>
       <c r="E15" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F15" s="27" t="n">
         <v>12</v>
@@ -3164,13 +3164,13 @@
         <v/>
       </c>
       <c r="C18" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>29</v>
       </c>
       <c r="E18" s="27" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F18" s="27" t="n">
         <v>10</v>
@@ -3219,13 +3219,13 @@
         <v/>
       </c>
       <c r="C19" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>32</v>
       </c>
       <c r="E19" s="27" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F19" s="27" t="n">
         <v>9</v>
@@ -3333,13 +3333,13 @@
         <v/>
       </c>
       <c r="C21" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>28</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F21" s="27" t="n">
         <v>13</v>
@@ -3388,13 +3388,13 @@
         <v/>
       </c>
       <c r="C22" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="27" t="n">
         <v>34</v>
       </c>
       <c r="E22" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F22" s="27" t="n">
         <v>10</v>
@@ -3553,13 +3553,13 @@
         <v/>
       </c>
       <c r="C25" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D25" s="27" t="n">
         <v>35</v>
       </c>
       <c r="E25" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F25" s="27" t="n">
         <v>11</v>
@@ -3608,13 +3608,13 @@
         <v/>
       </c>
       <c r="C26" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E26" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F26" s="27" t="n">
         <v>9</v>
@@ -3663,13 +3663,13 @@
         <v/>
       </c>
       <c r="C27" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" s="27" t="n">
         <v>36</v>
       </c>
       <c r="E27" s="27" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F27" s="27" t="n">
         <v>9</v>
@@ -3718,13 +3718,13 @@
         <v/>
       </c>
       <c r="C28" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="27" t="n">
         <v>36</v>
       </c>
       <c r="E28" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F28" s="27" t="n">
         <v>11</v>
@@ -3773,13 +3773,13 @@
         <v/>
       </c>
       <c r="C29" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" s="27" t="n">
         <v>36</v>
       </c>
       <c r="E29" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F29" s="27" t="n">
         <v>11</v>
@@ -3938,13 +3938,13 @@
         <v/>
       </c>
       <c r="C32" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D32" s="27" t="n">
         <v>29</v>
       </c>
       <c r="E32" s="27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F32" s="27" t="n">
         <v>9</v>
@@ -3993,13 +3993,13 @@
         <v/>
       </c>
       <c r="C33" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D33" s="27" t="n">
         <v>34</v>
       </c>
       <c r="E33" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F33" s="27" t="n">
         <v>12</v>
@@ -4048,13 +4048,13 @@
         <v/>
       </c>
       <c r="C34" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E34" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F34" s="27" t="n">
         <v>12</v>
@@ -4158,13 +4158,13 @@
         <v/>
       </c>
       <c r="C36" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" s="27" t="n">
         <v>28</v>
       </c>
       <c r="E36" s="27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F36" s="27" t="n">
         <v>9</v>
@@ -4323,13 +4323,13 @@
         <v/>
       </c>
       <c r="C39" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D39" s="27" t="n">
         <v>30</v>
       </c>
       <c r="E39" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F39" s="27" t="n">
         <v>9</v>
@@ -4378,13 +4378,13 @@
         <v/>
       </c>
       <c r="C40" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D40" s="27" t="n">
         <v>28</v>
       </c>
       <c r="E40" s="27" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F40" s="27" t="n">
         <v>13</v>
@@ -4433,13 +4433,13 @@
         <v/>
       </c>
       <c r="C41" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D41" s="27" t="n">
         <v>28</v>
       </c>
       <c r="E41" s="27" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F41" s="27" t="n">
         <v>10</v>
@@ -4488,13 +4488,13 @@
         <v/>
       </c>
       <c r="C42" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D42" s="27" t="n">
         <v>33</v>
       </c>
       <c r="E42" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F42" s="27" t="n">
         <v>13</v>
@@ -4543,13 +4543,13 @@
         <v/>
       </c>
       <c r="C43" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D43" s="27" t="n">
         <v>36</v>
       </c>
       <c r="E43" s="27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F43" s="27" t="n">
         <v>13</v>
@@ -4708,13 +4708,13 @@
         <v/>
       </c>
       <c r="C46" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D46" s="27" t="n">
         <v>31</v>
       </c>
       <c r="E46" s="27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F46" s="27" t="n">
         <v>9</v>
@@ -4763,13 +4763,13 @@
         <v/>
       </c>
       <c r="C47" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" s="27" t="n">
         <v>34</v>
       </c>
       <c r="E47" s="27" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F47" s="27" t="n">
         <v>12</v>
@@ -4818,13 +4818,13 @@
         <v/>
       </c>
       <c r="C48" s="27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" s="27" t="n">
         <v>33</v>
       </c>
       <c r="E48" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F48" s="27" t="n">
         <v>11</v>

</xml_diff>